<commit_message>
update Dex: DexGrasp Anything and Dexonomy leaderboards added; New models: Add ACT, KODex, KOROL, K-UBM, KAN-We-Flow, and X-DP3 to Adroit and DexArt; Add MP1 and AdaFlow to Adroit; Add the Dexonomy model to Dexonomy; Add KPGrasp to DexGrasp Anything and Dexonomy.
</commit_message>
<xml_diff>
--- a/assets/dex/raw/Dexterous Manipulation SOTA Leaderboard.xlsx
+++ b/assets/dex/raw/Dexterous Manipulation SOTA Leaderboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\E-AI\Sota Web\Evo-SOTA.io\assets\dex\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AD6BC04-8D4F-421E-858A-DC1FAFDA038B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A87839DE-B848-4878-B09E-412B72FA830B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4240" yWindow="640" windowWidth="28040" windowHeight="15800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="262">
   <si>
     <r>
       <t xml:space="preserve">Paper Link: </t>
@@ -974,105 +974,339 @@
     <t>https://jiaxin-lu.github.io/ugg/</t>
   </si>
   <si>
+    <t>DexGrasp Anything: Towards Universal Robotic Dexterous Grasping with Physics Awareness</t>
+  </si>
+  <si>
+    <t>EFF-Grasp: Energy-Field Flow Matching for Physics-Aware Dexterous Grasp Generation</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2603.16151</t>
+  </si>
+  <si>
+    <t>https://ieeexplore.ieee.org/document/9811666</t>
+  </si>
+  <si>
+    <t>FFHNet: Generating Multi-Fingered Robotic Grasps for Unknown Objects in Real-time</t>
+  </si>
+  <si>
+    <t>https://github.com/qqianfeng/FFHNet</t>
+  </si>
+  <si>
+    <t>DexDiffuser: Generating Dexterous Grasps with Diffusion Models</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2402.02989</t>
+  </si>
+  <si>
+    <t>https://yulihn.github.io/DexDiffuser_page/</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2605.13117v1</t>
+  </si>
+  <si>
+    <t>SECOND-Grasp: Semantic Contact-guided Dexterous Grasping</t>
+  </si>
+  <si>
+    <t>UniGraspTransformer: Simplified Policy Distillation for Scalable Dexterous Robotic Grasping</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2412.02699</t>
+  </si>
+  <si>
+    <t>https://dexhand.github.io/UniGraspTransformer/</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2509.22149</t>
+  </si>
+  <si>
+    <t>DemoGrasp: Universal Dexterous Grasping from a Single Demonstration</t>
+  </si>
+  <si>
+    <t>https://beingbeyond.github.io/DemoGrasp/</t>
+  </si>
+  <si>
+    <t>SAT</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Structural Action Transformer for 3D Dexterous Manipulation</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2603.03960</t>
+  </si>
+  <si>
+    <t>Origin</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>HPT</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>UniAct</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Scaling Proprioceptive-Visual Learning with Heterogeneous Pre-trained Transformers</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2409.20537</t>
+  </si>
+  <si>
+    <t>https://liruiw.github.io/hpt/</t>
+  </si>
+  <si>
+    <t>Reproduced by SAT</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Universal Actions for Enhanced Embodied Foundation Models</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2501.10105</t>
+  </si>
+  <si>
+    <t>https://2toinf.github.io/UniAct/</t>
+  </si>
+  <si>
+    <t>Learning Fine-Grained Bimanual Manipulation with Low-Cost Hardware</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>ACT</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>-</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Reproduced by K-UBM</t>
+  </si>
+  <si>
+    <t>Reproduced by K-UBM</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Optimized by K-UBM</t>
+  </si>
+  <si>
+    <t>Optimized by K-UBM</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>KODex</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>On the Utility of Koopman Operator Theory in Learning Dexterous Manipulation Skills</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Origin</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2304.13705</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>KOROL</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>KOROL: Learning Visualizable Object Feature with Koopman Operator Rollout for Manipulation</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>K-UBM</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Going with the Flow: Koopman Behavioral Models as Pseudo Planners for Visuo-Motor Dexterity</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>GSR</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Setting</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Source</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Proof</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>DexGrasp Anything</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>OSR</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>CDC</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>PD</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Div.</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dexonomy</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Reproduced by KPGrasp</t>
+  </si>
+  <si>
+    <t>Reproduced by KPGrasp</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dexonomy: Synthesizing All Dexterous Grasp Types in a Grasp Taxonomy</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Paper Link: https://arxiv.org/abs/2504.18829</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Project Link: https://pku-epic.github.io/Dexonomy/</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>with classifier</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>KPGrasp</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>KPGrasp: Scalable Keypoint Flow Matching for Dexterous Grasp Generation</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>GSR.(avg)</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pen.(avg)</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://dexgraspanything.github.io/</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Project Link: https://dexgraspanything.github.io/</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
     <t>https://arxiv.org/abs/2503.08257</t>
-  </si>
-  <si>
-    <t>DexGrasp Anything: Towards Universal Robotic Dexterous Grasping with Physics Awareness</t>
-  </si>
-  <si>
-    <t>https://dexgraspanything.github.io/</t>
-  </si>
-  <si>
-    <t>EFF-Grasp: Energy-Field Flow Matching for Physics-Aware Dexterous Grasp Generation</t>
-  </si>
-  <si>
-    <t>https://arxiv.org/abs/2603.16151</t>
-  </si>
-  <si>
-    <t>https://ieeexplore.ieee.org/document/9811666</t>
-  </si>
-  <si>
-    <t>FFHNet: Generating Multi-Fingered Robotic Grasps for Unknown Objects in Real-time</t>
-  </si>
-  <si>
-    <t>https://github.com/qqianfeng/FFHNet</t>
-  </si>
-  <si>
-    <t>DexDiffuser: Generating Dexterous Grasps with Diffusion Models</t>
-  </si>
-  <si>
-    <t>https://arxiv.org/abs/2402.02989</t>
-  </si>
-  <si>
-    <t>https://yulihn.github.io/DexDiffuser_page/</t>
-  </si>
-  <si>
-    <t>https://arxiv.org/abs/2605.13117v1</t>
-  </si>
-  <si>
-    <t>SECOND-Grasp: Semantic Contact-guided Dexterous Grasping</t>
-  </si>
-  <si>
-    <t>UniGraspTransformer: Simplified Policy Distillation for Scalable Dexterous Robotic Grasping</t>
-  </si>
-  <si>
-    <t>https://arxiv.org/abs/2412.02699</t>
-  </si>
-  <si>
-    <t>https://dexhand.github.io/UniGraspTransformer/</t>
-  </si>
-  <si>
-    <t>https://arxiv.org/abs/2509.22149</t>
-  </si>
-  <si>
-    <t>DemoGrasp: Universal Dexterous Grasping from a Single Demonstration</t>
-  </si>
-  <si>
-    <t>https://beingbeyond.github.io/DemoGrasp/</t>
-  </si>
-  <si>
-    <t>SAT</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>Structural Action Transformer for 3D Dexterous Manipulation</t>
-  </si>
-  <si>
-    <t>https://arxiv.org/abs/2603.03960</t>
-  </si>
-  <si>
-    <t>Origin</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>HPT</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>UniAct</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>Scaling Proprioceptive-Visual Learning with Heterogeneous Pre-trained Transformers</t>
-  </si>
-  <si>
-    <t>https://arxiv.org/abs/2409.20537</t>
-  </si>
-  <si>
-    <t>https://liruiw.github.io/hpt/</t>
-  </si>
-  <si>
-    <t>Reproduced by SAT</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>Universal Actions for Enhanced Embodied Foundation Models</t>
-  </si>
-  <si>
-    <t>https://arxiv.org/abs/2501.10105</t>
-  </si>
-  <si>
-    <t>https://2toinf.github.io/UniAct/</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Paper page: https://arxiv.org/abs/2503.08257</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>KAN-We-Flow</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>KAN We Flow? Advancing Robotic Manipulation with 3D Flow Matching via KAN &amp; RWKV</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>X-DP3</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>X-Imitator: Spatial-Aware Imitation Learning via Bidirectional Action-Pose Interaction</t>
+  </si>
+  <si>
+    <t>MP1: MeanFlow Tames Policy Learning in 1-step for Robotic Manipulation</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>MP1</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>AdaFlow</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>AdaFlow: Imitation Learning with Variance-Adaptive Flow-Based Policies</t>
+  </si>
+  <si>
+    <t>Reproduced by KAN-We-Flow</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2303.13446</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://github.com/GT-STAR-Lab/KODex</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2407.00548</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://github.com/hychen-naza/KOROL</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2602.07413</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://github.com/GT-STAR-Lab/K-UBM</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2504.18829</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://github.com/JYChen18/Dexonomy</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2606.09314</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2602.01115</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2605.12162</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2507.10543</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://github.com/LogSSim/MP1</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2402.04292</t>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1156,7 +1390,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -1377,12 +1611,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1444,6 +1687,30 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1476,9 +1743,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3143,143 +3407,186 @@
     <col min="45" max="45" width="14" style="13" customWidth="1"/>
     <col min="46" max="46" width="14" style="17" customWidth="1"/>
     <col min="47" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="14" style="13" customWidth="1"/>
-    <col min="53" max="111" width="14" customWidth="1"/>
+    <col min="52" max="52" width="14" style="17" customWidth="1"/>
+    <col min="53" max="53" width="14" style="24" customWidth="1"/>
+    <col min="54" max="56" width="14" customWidth="1"/>
+    <col min="57" max="57" width="14" style="13" customWidth="1"/>
+    <col min="58" max="64" width="14" customWidth="1"/>
+    <col min="65" max="65" width="14" style="13" customWidth="1"/>
+    <col min="66" max="111" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:111" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="34" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="27" t="s">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="27" t="s">
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="36"/>
+      <c r="N1" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="O1" s="27"/>
-      <c r="P1" s="27"/>
-      <c r="Q1" s="27"/>
-      <c r="R1" s="27"/>
-      <c r="S1" s="27"/>
-      <c r="T1" s="27"/>
-      <c r="U1" s="28"/>
-      <c r="V1" s="29" t="s">
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
+      <c r="R1" s="35"/>
+      <c r="S1" s="35"/>
+      <c r="T1" s="35"/>
+      <c r="U1" s="36"/>
+      <c r="V1" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="W1" s="29"/>
-      <c r="X1" s="29"/>
-      <c r="Y1" s="29"/>
-      <c r="Z1" s="29"/>
-      <c r="AA1" s="29"/>
-      <c r="AB1" s="29"/>
-      <c r="AC1" s="29"/>
-      <c r="AD1" s="29"/>
-      <c r="AE1" s="29"/>
-      <c r="AF1" s="29"/>
-      <c r="AG1" s="29"/>
-      <c r="AH1" s="29"/>
-      <c r="AI1" s="29"/>
-      <c r="AJ1" s="29"/>
-      <c r="AK1" s="29"/>
-      <c r="AL1" s="29"/>
-      <c r="AM1" s="29"/>
-      <c r="AN1" s="29"/>
-      <c r="AO1" s="29"/>
-      <c r="AP1" s="29"/>
-      <c r="AQ1" s="29"/>
-      <c r="AR1" s="29"/>
-      <c r="AS1" s="29"/>
-      <c r="AT1" s="21" t="s">
+      <c r="W1" s="37"/>
+      <c r="X1" s="37"/>
+      <c r="Y1" s="37"/>
+      <c r="Z1" s="37"/>
+      <c r="AA1" s="37"/>
+      <c r="AB1" s="37"/>
+      <c r="AC1" s="37"/>
+      <c r="AD1" s="37"/>
+      <c r="AE1" s="37"/>
+      <c r="AF1" s="37"/>
+      <c r="AG1" s="37"/>
+      <c r="AH1" s="37"/>
+      <c r="AI1" s="37"/>
+      <c r="AJ1" s="37"/>
+      <c r="AK1" s="37"/>
+      <c r="AL1" s="37"/>
+      <c r="AM1" s="37"/>
+      <c r="AN1" s="37"/>
+      <c r="AO1" s="37"/>
+      <c r="AP1" s="37"/>
+      <c r="AQ1" s="37"/>
+      <c r="AR1" s="37"/>
+      <c r="AS1" s="37"/>
+      <c r="AT1" s="29" t="s">
         <v>134</v>
       </c>
-      <c r="AU1" s="22"/>
-      <c r="AV1" s="22"/>
-      <c r="AW1" s="22"/>
-      <c r="AX1" s="22"/>
-      <c r="AY1" s="22"/>
-      <c r="AZ1" s="22"/>
+      <c r="AU1" s="30"/>
+      <c r="AV1" s="30"/>
+      <c r="AW1" s="30"/>
+      <c r="AX1" s="30"/>
+      <c r="AY1" s="30"/>
+      <c r="AZ1" s="30"/>
+      <c r="BA1" s="25" t="s">
+        <v>219</v>
+      </c>
+      <c r="BB1" s="25"/>
+      <c r="BC1" s="25"/>
+      <c r="BD1" s="25"/>
+      <c r="BE1" s="25"/>
+      <c r="BF1" s="25" t="s">
+        <v>224</v>
+      </c>
+      <c r="BG1" s="25"/>
+      <c r="BH1" s="25"/>
+      <c r="BI1" s="25"/>
+      <c r="BJ1" s="25"/>
+      <c r="BK1" s="25"/>
+      <c r="BL1" s="25"/>
+      <c r="BM1" s="25"/>
     </row>
     <row r="2" spans="1:111" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="26"/>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="30" t="s">
+      <c r="A2" s="34"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="27" t="s">
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="38"/>
+      <c r="J2" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
-      <c r="N2" s="27" t="s">
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="O2" s="27"/>
-      <c r="P2" s="27"/>
-      <c r="Q2" s="27"/>
-      <c r="R2" s="27" t="s">
+      <c r="O2" s="35"/>
+      <c r="P2" s="35"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="S2" s="27"/>
-      <c r="T2" s="27"/>
-      <c r="U2" s="27"/>
-      <c r="V2" s="29" t="s">
+      <c r="S2" s="35"/>
+      <c r="T2" s="35"/>
+      <c r="U2" s="35"/>
+      <c r="V2" s="37" t="s">
         <v>136</v>
       </c>
-      <c r="W2" s="29"/>
-      <c r="X2" s="29"/>
-      <c r="Y2" s="29"/>
-      <c r="Z2" s="29"/>
-      <c r="AA2" s="29"/>
-      <c r="AB2" s="29"/>
-      <c r="AC2" s="29"/>
-      <c r="AD2" s="29"/>
-      <c r="AE2" s="29"/>
-      <c r="AF2" s="29"/>
-      <c r="AG2" s="29"/>
-      <c r="AH2" s="29" t="s">
+      <c r="W2" s="37"/>
+      <c r="X2" s="37"/>
+      <c r="Y2" s="37"/>
+      <c r="Z2" s="37"/>
+      <c r="AA2" s="37"/>
+      <c r="AB2" s="37"/>
+      <c r="AC2" s="37"/>
+      <c r="AD2" s="37"/>
+      <c r="AE2" s="37"/>
+      <c r="AF2" s="37"/>
+      <c r="AG2" s="37"/>
+      <c r="AH2" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="AI2" s="29"/>
-      <c r="AJ2" s="29"/>
-      <c r="AK2" s="29"/>
-      <c r="AL2" s="29"/>
-      <c r="AM2" s="29"/>
-      <c r="AN2" s="29"/>
-      <c r="AO2" s="29"/>
-      <c r="AP2" s="29"/>
-      <c r="AQ2" s="29"/>
-      <c r="AR2" s="29"/>
-      <c r="AS2" s="31"/>
-      <c r="AT2" s="23" t="s">
+      <c r="AI2" s="37"/>
+      <c r="AJ2" s="37"/>
+      <c r="AK2" s="37"/>
+      <c r="AL2" s="37"/>
+      <c r="AM2" s="37"/>
+      <c r="AN2" s="37"/>
+      <c r="AO2" s="37"/>
+      <c r="AP2" s="37"/>
+      <c r="AQ2" s="37"/>
+      <c r="AR2" s="37"/>
+      <c r="AS2" s="39"/>
+      <c r="AT2" s="31" t="s">
         <v>138</v>
       </c>
-      <c r="AU2" s="24"/>
-      <c r="AV2" s="24"/>
-      <c r="AW2" s="25"/>
-      <c r="AX2" s="23" t="s">
+      <c r="AU2" s="32"/>
+      <c r="AV2" s="32"/>
+      <c r="AW2" s="33"/>
+      <c r="AX2" s="31" t="s">
         <v>137</v>
       </c>
-      <c r="AY2" s="24"/>
-      <c r="AZ2" s="25"/>
+      <c r="AY2" s="32"/>
+      <c r="AZ2" s="33"/>
+      <c r="BA2" s="26" t="s">
+        <v>236</v>
+      </c>
+      <c r="BB2" s="27"/>
+      <c r="BC2" s="26" t="s">
+        <v>238</v>
+      </c>
+      <c r="BD2" s="27"/>
+      <c r="BE2" s="28"/>
+      <c r="BF2" s="26" t="s">
+        <v>229</v>
+      </c>
+      <c r="BG2" s="27"/>
+      <c r="BH2" s="27"/>
+      <c r="BI2" s="28"/>
+      <c r="BJ2" s="26" t="s">
+        <v>228</v>
+      </c>
+      <c r="BK2" s="27"/>
+      <c r="BL2" s="27"/>
+      <c r="BM2" s="28"/>
     </row>
     <row r="3" spans="1:111" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
@@ -3435,22 +3742,48 @@
       <c r="AY3" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="AZ3" s="14" t="s">
+      <c r="AZ3" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="BA3" s="2"/>
-      <c r="BB3" s="2"/>
-      <c r="BC3" s="2"/>
-      <c r="BD3" s="2"/>
-      <c r="BE3" s="2"/>
-      <c r="BF3" s="2"/>
-      <c r="BG3" s="2"/>
-      <c r="BH3" s="2"/>
-      <c r="BI3" s="2"/>
-      <c r="BJ3" s="2"/>
-      <c r="BK3" s="2"/>
-      <c r="BL3" s="2"/>
-      <c r="BM3" s="2"/>
+      <c r="BA3" s="23" t="s">
+        <v>233</v>
+      </c>
+      <c r="BB3" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="BC3" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="BD3" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="BE3" s="14" t="s">
+        <v>218</v>
+      </c>
+      <c r="BF3" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="BG3" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="BH3" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="BI3" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="BJ3" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="BK3" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="BL3" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="BM3" s="14" t="s">
+        <v>218</v>
+      </c>
       <c r="BN3" s="2"/>
       <c r="BO3" s="2"/>
       <c r="BP3" s="2"/>
@@ -4319,7 +4652,7 @@
       <c r="U16" s="1"/>
       <c r="AS16" s="14"/>
     </row>
-    <row r="17" spans="1:52" ht="78" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:64" ht="78" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>115</v>
       </c>
@@ -4375,7 +4708,7 @@
       <c r="U17" s="1"/>
       <c r="AS17" s="14"/>
     </row>
-    <row r="18" spans="1:52" ht="102" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:64" ht="102" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>117</v>
       </c>
@@ -4464,7 +4797,7 @@
       </c>
       <c r="AS18" s="14"/>
     </row>
-    <row r="19" spans="1:52" ht="76.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:64" ht="76.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>119</v>
       </c>
@@ -4553,7 +4886,7 @@
       </c>
       <c r="AS19" s="14"/>
     </row>
-    <row r="20" spans="1:52" ht="88.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:64" ht="88.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
         <v>121</v>
       </c>
@@ -4589,7 +4922,7 @@
       <c r="U20" s="1"/>
       <c r="AS20" s="14"/>
     </row>
-    <row r="21" spans="1:52" ht="91" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:64" ht="91" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
         <v>123</v>
       </c>
@@ -4632,7 +4965,7 @@
       <c r="U21" s="1"/>
       <c r="AS21" s="14"/>
     </row>
-    <row r="22" spans="1:52" ht="65" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:64" ht="65" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>139</v>
       </c>
@@ -4698,9 +5031,9 @@
       <c r="AY22" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="AZ22" s="16"/>
-    </row>
-    <row r="23" spans="1:52" ht="78" x14ac:dyDescent="0.3">
+      <c r="AZ22" s="18"/>
+    </row>
+    <row r="23" spans="1:64" ht="78" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>140</v>
       </c>
@@ -4772,9 +5105,18 @@
       <c r="AY23" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="AZ23" s="16"/>
-    </row>
-    <row r="24" spans="1:52" ht="130" x14ac:dyDescent="0.3">
+      <c r="AZ23" s="18"/>
+      <c r="BA23" s="24">
+        <v>19.5</v>
+      </c>
+      <c r="BB23">
+        <v>31.2</v>
+      </c>
+      <c r="BD23" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="24" spans="1:64" ht="130" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>135</v>
       </c>
@@ -4846,9 +5188,36 @@
       <c r="AY24" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="AZ24" s="16"/>
-    </row>
-    <row r="25" spans="1:52" ht="65" x14ac:dyDescent="0.3">
+      <c r="AZ24" s="18"/>
+      <c r="BA24" s="24">
+        <v>25.4</v>
+      </c>
+      <c r="BB24">
+        <v>29.3</v>
+      </c>
+      <c r="BD24" t="s">
+        <v>225</v>
+      </c>
+      <c r="BF24">
+        <v>24.5</v>
+      </c>
+      <c r="BG24">
+        <v>73.2</v>
+      </c>
+      <c r="BH24">
+        <v>15.6</v>
+      </c>
+      <c r="BI24">
+        <v>11.6</v>
+      </c>
+      <c r="BJ24">
+        <v>28</v>
+      </c>
+      <c r="BL24" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="25" spans="1:64" ht="65" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>141</v>
       </c>
@@ -4920,9 +5289,18 @@
       <c r="AY25" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="AZ25" s="16"/>
-    </row>
-    <row r="26" spans="1:52" ht="39" x14ac:dyDescent="0.3">
+      <c r="AZ25" s="18"/>
+      <c r="BA25" s="24">
+        <v>37.1</v>
+      </c>
+      <c r="BB25">
+        <v>30.8</v>
+      </c>
+      <c r="BD25" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="26" spans="1:64" ht="39" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>142</v>
       </c>
@@ -4994,23 +5372,32 @@
       <c r="AY26" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="AZ26" s="16"/>
-    </row>
-    <row r="27" spans="1:52" ht="104" x14ac:dyDescent="0.3">
+      <c r="AZ26" s="18"/>
+      <c r="BA26" s="24">
+        <v>44.7</v>
+      </c>
+      <c r="BB26">
+        <v>25.5</v>
+      </c>
+      <c r="BD26" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="27" spans="1:64" ht="104" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>151</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C27" s="2">
         <v>2025.03</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>170</v>
+        <v>237</v>
       </c>
       <c r="E27" s="19" t="s">
-        <v>172</v>
+        <v>235</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
@@ -5068,20 +5455,47 @@
       <c r="AY27" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="AZ27" s="16"/>
-    </row>
-    <row r="28" spans="1:52" ht="91" x14ac:dyDescent="0.3">
+      <c r="AZ27" s="18"/>
+      <c r="BA27" s="24">
+        <v>58.5</v>
+      </c>
+      <c r="BB27">
+        <v>21.2</v>
+      </c>
+      <c r="BD27" t="s">
+        <v>225</v>
+      </c>
+      <c r="BF27">
+        <v>21.8</v>
+      </c>
+      <c r="BG27">
+        <v>72.2</v>
+      </c>
+      <c r="BH27">
+        <v>11</v>
+      </c>
+      <c r="BI27">
+        <v>14.2</v>
+      </c>
+      <c r="BJ27">
+        <v>23.3</v>
+      </c>
+      <c r="BL27" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="28" spans="1:64" ht="91" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>149</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C28" s="2">
         <v>2026.03</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
@@ -5140,23 +5554,23 @@
       <c r="AY28" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="AZ28" s="16"/>
-    </row>
-    <row r="29" spans="1:52" ht="91" x14ac:dyDescent="0.3">
+      <c r="AZ28" s="18"/>
+    </row>
+    <row r="29" spans="1:64" ht="91" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>153</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C29" s="2">
         <v>2022.05</v>
       </c>
       <c r="D29" s="19" t="s">
+        <v>173</v>
+      </c>
+      <c r="E29" s="19" t="s">
         <v>175</v>
-      </c>
-      <c r="E29" s="19" t="s">
-        <v>177</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -5208,23 +5622,23 @@
       <c r="AY29" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="AZ29" s="16"/>
-    </row>
-    <row r="30" spans="1:52" ht="65" x14ac:dyDescent="0.3">
+      <c r="AZ29" s="18"/>
+    </row>
+    <row r="30" spans="1:64" ht="65" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>143</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C30" s="2">
         <v>2024.02</v>
       </c>
       <c r="D30" s="19" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E30" s="19" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -5278,20 +5692,20 @@
       <c r="AY30" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="AZ30" s="16"/>
-    </row>
-    <row r="31" spans="1:52" ht="65" x14ac:dyDescent="0.3">
+      <c r="AZ30" s="18"/>
+    </row>
+    <row r="31" spans="1:64" ht="65" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>144</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C31" s="2">
         <v>2026.05</v>
       </c>
       <c r="D31" s="19" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
@@ -5346,23 +5760,23 @@
       <c r="AY31" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="AZ31" s="16"/>
-    </row>
-    <row r="32" spans="1:52" ht="78" x14ac:dyDescent="0.3">
+      <c r="AZ31" s="18"/>
+    </row>
+    <row r="32" spans="1:64" ht="78" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>147</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C32" s="2">
         <v>2024.12</v>
       </c>
       <c r="D32" s="19" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -5416,23 +5830,23 @@
       <c r="AY32" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="AZ32" s="16"/>
-    </row>
-    <row r="33" spans="1:52" ht="78" x14ac:dyDescent="0.3">
+      <c r="AZ32" s="18"/>
+    </row>
+    <row r="33" spans="1:64" ht="78" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>148</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C33" s="2">
         <v>2025.09</v>
       </c>
       <c r="D33" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="E33" s="19" t="s">
         <v>186</v>
-      </c>
-      <c r="E33" s="19" t="s">
-        <v>188</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -5486,159 +5900,606 @@
       <c r="AY33" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="AZ33" s="16"/>
-    </row>
-    <row r="34" spans="1:52" ht="52" x14ac:dyDescent="0.3">
+      <c r="AZ33" s="18"/>
+    </row>
+    <row r="34" spans="1:64" ht="52" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C34">
         <v>2026.03</v>
       </c>
       <c r="D34" s="19" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="E34" s="19"/>
       <c r="F34">
         <v>75</v>
       </c>
       <c r="L34" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="M34" s="1"/>
       <c r="R34">
         <v>73</v>
       </c>
       <c r="T34" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="U34" s="1"/>
       <c r="AS34" s="14"/>
     </row>
-    <row r="35" spans="1:52" ht="91" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:64" ht="91" x14ac:dyDescent="0.3">
       <c r="A35" s="20" t="s">
+        <v>191</v>
+      </c>
+      <c r="B35" s="4" t="s">
         <v>193</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>195</v>
       </c>
       <c r="C35">
         <v>2024.09</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="E35" s="19" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="F35">
         <v>45</v>
       </c>
       <c r="L35" s="20" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="M35" s="1"/>
       <c r="R35">
         <v>53</v>
       </c>
-      <c r="T35" s="32" t="s">
-        <v>198</v>
+      <c r="T35" s="21" t="s">
+        <v>196</v>
       </c>
       <c r="U35" s="1"/>
-      <c r="AR35" s="32"/>
+      <c r="AR35" s="21"/>
       <c r="AS35" s="14"/>
     </row>
-    <row r="36" spans="1:52" ht="65" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:64" ht="65" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C36">
         <v>2025.01</v>
       </c>
       <c r="D36" s="19" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="E36" s="19" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F36">
         <v>49</v>
       </c>
       <c r="L36" s="20" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="M36" s="1"/>
       <c r="R36">
         <v>55</v>
       </c>
-      <c r="T36" s="32" t="s">
-        <v>198</v>
+      <c r="T36" s="21" t="s">
+        <v>196</v>
       </c>
       <c r="U36" s="1"/>
       <c r="AS36" s="14"/>
     </row>
-    <row r="37" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:64" ht="78" x14ac:dyDescent="0.3">
+      <c r="A37" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C37">
+        <v>2023.04</v>
+      </c>
+      <c r="D37" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="F37">
+        <v>78.95</v>
+      </c>
+      <c r="G37">
+        <v>85</v>
+      </c>
+      <c r="H37">
+        <v>44.7</v>
+      </c>
+      <c r="I37">
+        <v>96.7</v>
+      </c>
+      <c r="J37">
+        <v>89.4</v>
+      </c>
+      <c r="K37" t="s">
+        <v>205</v>
+      </c>
+      <c r="L37" t="s">
+        <v>204</v>
+      </c>
       <c r="M37" s="1"/>
+      <c r="N37">
+        <v>92</v>
+      </c>
+      <c r="O37" t="s">
+        <v>202</v>
+      </c>
+      <c r="P37">
+        <v>78.7</v>
+      </c>
+      <c r="Q37">
+        <v>83.3</v>
+      </c>
+      <c r="R37">
+        <v>84.67</v>
+      </c>
+      <c r="S37" t="s">
+        <v>206</v>
+      </c>
+      <c r="T37" t="s">
+        <v>204</v>
+      </c>
       <c r="U37" s="1"/>
       <c r="AS37" s="14"/>
     </row>
-    <row r="38" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:64" ht="91" x14ac:dyDescent="0.3">
+      <c r="A38" s="20" t="s">
+        <v>207</v>
+      </c>
+      <c r="B38" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="C38">
+        <v>2023.03</v>
+      </c>
+      <c r="D38" s="22" t="s">
+        <v>248</v>
+      </c>
+      <c r="E38" t="s">
+        <v>249</v>
+      </c>
+      <c r="F38">
+        <v>86.5</v>
+      </c>
+      <c r="G38">
+        <v>62</v>
+      </c>
+      <c r="H38">
+        <v>96</v>
+      </c>
+      <c r="I38">
+        <v>100</v>
+      </c>
+      <c r="J38">
+        <v>88</v>
+      </c>
+      <c r="L38" t="s">
+        <v>209</v>
+      </c>
       <c r="M38" s="1"/>
+      <c r="N38">
+        <v>33.299999999999997</v>
+      </c>
+      <c r="O38" t="s">
+        <v>202</v>
+      </c>
+      <c r="P38">
+        <v>3.4</v>
+      </c>
+      <c r="Q38">
+        <v>80</v>
+      </c>
+      <c r="R38">
+        <v>38.9</v>
+      </c>
+      <c r="S38" t="s">
+        <v>205</v>
+      </c>
+      <c r="T38" t="s">
+        <v>204</v>
+      </c>
       <c r="U38" s="1"/>
       <c r="AS38" s="14"/>
     </row>
-    <row r="39" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:64" ht="78" x14ac:dyDescent="0.3">
+      <c r="A39" s="20" t="s">
+        <v>211</v>
+      </c>
+      <c r="B39" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="C39">
+        <v>2024.07</v>
+      </c>
+      <c r="D39" s="22" t="s">
+        <v>250</v>
+      </c>
+      <c r="E39" s="22" t="s">
+        <v>251</v>
+      </c>
+      <c r="F39">
+        <v>96.6</v>
+      </c>
+      <c r="G39">
+        <v>100</v>
+      </c>
+      <c r="H39">
+        <v>99.9</v>
+      </c>
+      <c r="I39">
+        <v>100</v>
+      </c>
+      <c r="J39">
+        <v>86.4</v>
+      </c>
+      <c r="L39" t="s">
+        <v>209</v>
+      </c>
       <c r="M39" s="1"/>
+      <c r="N39">
+        <v>71.3</v>
+      </c>
+      <c r="O39" t="s">
+        <v>202</v>
+      </c>
+      <c r="P39">
+        <v>53.1</v>
+      </c>
+      <c r="Q39">
+        <v>78.7</v>
+      </c>
+      <c r="R39">
+        <v>67.7</v>
+      </c>
+      <c r="S39" t="s">
+        <v>205</v>
+      </c>
+      <c r="T39" t="s">
+        <v>203</v>
+      </c>
       <c r="U39" s="1"/>
       <c r="AS39" s="14"/>
     </row>
-    <row r="40" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:64" ht="91" x14ac:dyDescent="0.3">
+      <c r="A40" s="20" t="s">
+        <v>213</v>
+      </c>
+      <c r="B40" s="20" t="s">
+        <v>214</v>
+      </c>
+      <c r="C40">
+        <v>2026.02</v>
+      </c>
+      <c r="D40" s="22" t="s">
+        <v>252</v>
+      </c>
+      <c r="E40" s="22" t="s">
+        <v>253</v>
+      </c>
+      <c r="F40">
+        <v>76.875</v>
+      </c>
+      <c r="G40">
+        <v>92.5</v>
+      </c>
+      <c r="H40">
+        <v>57</v>
+      </c>
+      <c r="I40">
+        <v>89</v>
+      </c>
+      <c r="J40">
+        <v>69</v>
+      </c>
+      <c r="L40" t="s">
+        <v>209</v>
+      </c>
       <c r="M40" s="1"/>
+      <c r="N40">
+        <v>58</v>
+      </c>
+      <c r="O40" t="s">
+        <v>202</v>
+      </c>
+      <c r="P40">
+        <v>76</v>
+      </c>
+      <c r="Q40">
+        <v>76.5</v>
+      </c>
+      <c r="R40">
+        <v>70.17</v>
+      </c>
+      <c r="T40" t="s">
+        <v>209</v>
+      </c>
       <c r="U40" s="1"/>
       <c r="AS40" s="14"/>
     </row>
-    <row r="41" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:64" ht="65" x14ac:dyDescent="0.3">
+      <c r="A41" s="20" t="s">
+        <v>224</v>
+      </c>
+      <c r="B41" s="20" t="s">
+        <v>227</v>
+      </c>
+      <c r="C41">
+        <v>2025.04</v>
+      </c>
+      <c r="D41" s="22" t="s">
+        <v>254</v>
+      </c>
+      <c r="E41" t="s">
+        <v>255</v>
+      </c>
       <c r="M41" s="1"/>
       <c r="U41" s="1"/>
       <c r="AS41" s="14"/>
-    </row>
-    <row r="42" spans="1:52" x14ac:dyDescent="0.3">
+      <c r="BF41">
+        <v>63.9</v>
+      </c>
+      <c r="BG41">
+        <v>91.3</v>
+      </c>
+      <c r="BH41">
+        <v>13.9</v>
+      </c>
+      <c r="BI41">
+        <v>8.6</v>
+      </c>
+      <c r="BJ41">
+        <v>25.7</v>
+      </c>
+      <c r="BK41" t="s">
+        <v>230</v>
+      </c>
+      <c r="BL41" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="42" spans="1:64" ht="78" x14ac:dyDescent="0.3">
+      <c r="A42" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="B42" s="20" t="s">
+        <v>232</v>
+      </c>
+      <c r="C42">
+        <v>2026.06</v>
+      </c>
+      <c r="D42" s="22" t="s">
+        <v>256</v>
+      </c>
       <c r="M42" s="1"/>
       <c r="U42" s="1"/>
       <c r="AS42" s="14"/>
-    </row>
-    <row r="43" spans="1:52" x14ac:dyDescent="0.3">
+      <c r="BA42" s="24">
+        <v>63.8</v>
+      </c>
+      <c r="BB42">
+        <v>12.9</v>
+      </c>
+      <c r="BD42" t="s">
+        <v>209</v>
+      </c>
+      <c r="BF42">
+        <v>76.3</v>
+      </c>
+      <c r="BG42">
+        <v>97.3</v>
+      </c>
+      <c r="BH42">
+        <v>5.6</v>
+      </c>
+      <c r="BI42">
+        <v>2.4</v>
+      </c>
+      <c r="BJ42">
+        <v>23.3</v>
+      </c>
+      <c r="BL42" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="43" spans="1:64" ht="91" x14ac:dyDescent="0.3">
+      <c r="A43" s="20" t="s">
+        <v>239</v>
+      </c>
+      <c r="B43" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="C43">
+        <v>2026.02</v>
+      </c>
+      <c r="D43" s="22" t="s">
+        <v>257</v>
+      </c>
+      <c r="F43">
+        <v>83.67</v>
+      </c>
+      <c r="G43">
+        <v>68</v>
+      </c>
+      <c r="H43">
+        <v>83</v>
+      </c>
+      <c r="I43">
+        <v>100</v>
+      </c>
+      <c r="J43" t="s">
+        <v>202</v>
+      </c>
+      <c r="L43" t="s">
+        <v>145</v>
+      </c>
       <c r="M43" s="1"/>
+      <c r="N43">
+        <v>85</v>
+      </c>
+      <c r="O43">
+        <v>42.5</v>
+      </c>
+      <c r="P43">
+        <v>82</v>
+      </c>
+      <c r="Q43">
+        <v>35</v>
+      </c>
+      <c r="R43">
+        <v>61.125</v>
+      </c>
+      <c r="T43" t="s">
+        <v>145</v>
+      </c>
       <c r="U43" s="1"/>
       <c r="AS43" s="14"/>
     </row>
-    <row r="44" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:64" ht="91" x14ac:dyDescent="0.3">
+      <c r="A44" s="20" t="s">
+        <v>241</v>
+      </c>
+      <c r="B44" s="20" t="s">
+        <v>242</v>
+      </c>
+      <c r="C44">
+        <v>2026.05</v>
+      </c>
+      <c r="D44" s="22" t="s">
+        <v>258</v>
+      </c>
+      <c r="F44">
+        <v>71.17</v>
+      </c>
+      <c r="G44">
+        <v>45.3</v>
+      </c>
+      <c r="H44">
+        <v>68.5</v>
+      </c>
+      <c r="I44">
+        <v>99.7</v>
+      </c>
+      <c r="J44" t="s">
+        <v>202</v>
+      </c>
+      <c r="L44" t="s">
+        <v>145</v>
+      </c>
       <c r="M44" s="1"/>
+      <c r="N44">
+        <v>74.7</v>
+      </c>
+      <c r="O44">
+        <v>40.6</v>
+      </c>
+      <c r="P44">
+        <v>64.400000000000006</v>
+      </c>
+      <c r="Q44">
+        <v>58.2</v>
+      </c>
+      <c r="R44">
+        <v>59.475000000000001</v>
+      </c>
+      <c r="T44" t="s">
+        <v>145</v>
+      </c>
       <c r="U44" s="1"/>
       <c r="AS44" s="14"/>
     </row>
-    <row r="45" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:64" ht="65" x14ac:dyDescent="0.3">
+      <c r="A45" s="20" t="s">
+        <v>244</v>
+      </c>
+      <c r="B45" s="20" t="s">
+        <v>243</v>
+      </c>
+      <c r="C45">
+        <v>2025.07</v>
+      </c>
+      <c r="D45" s="22" t="s">
+        <v>259</v>
+      </c>
+      <c r="E45" t="s">
+        <v>260</v>
+      </c>
+      <c r="F45">
+        <v>75.67</v>
+      </c>
+      <c r="G45">
+        <v>58</v>
+      </c>
+      <c r="H45">
+        <v>69</v>
+      </c>
+      <c r="I45">
+        <v>100</v>
+      </c>
+      <c r="J45" t="s">
+        <v>202</v>
+      </c>
+      <c r="L45" t="s">
+        <v>247</v>
+      </c>
       <c r="M45" s="1"/>
       <c r="U45" s="1"/>
       <c r="AS45" s="14"/>
     </row>
-    <row r="46" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:64" ht="78" x14ac:dyDescent="0.3">
+      <c r="A46" s="20" t="s">
+        <v>245</v>
+      </c>
+      <c r="B46" s="20" t="s">
+        <v>246</v>
+      </c>
+      <c r="C46">
+        <v>2024.02</v>
+      </c>
+      <c r="D46" s="22" t="s">
+        <v>261</v>
+      </c>
+      <c r="F46">
+        <v>30</v>
+      </c>
+      <c r="G46">
+        <v>18</v>
+      </c>
+      <c r="H46">
+        <v>27</v>
+      </c>
+      <c r="I46">
+        <v>45</v>
+      </c>
+      <c r="J46" t="s">
+        <v>202</v>
+      </c>
+      <c r="L46" t="s">
+        <v>247</v>
+      </c>
       <c r="M46" s="1"/>
       <c r="U46" s="1"/>
       <c r="AS46" s="14"/>
     </row>
-    <row r="47" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:64" x14ac:dyDescent="0.3">
       <c r="M47" s="1"/>
       <c r="U47" s="1"/>
       <c r="AS47" s="14"/>
     </row>
-    <row r="48" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:64" x14ac:dyDescent="0.3">
       <c r="M48" s="1"/>
       <c r="U48" s="1"/>
       <c r="AS48" s="14"/>
@@ -6364,7 +7225,7 @@
       <c r="AS192" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="19">
     <mergeCell ref="AT1:AZ1"/>
     <mergeCell ref="AT2:AW2"/>
     <mergeCell ref="AX2:AZ2"/>
@@ -6378,6 +7239,12 @@
     <mergeCell ref="AH2:AS2"/>
     <mergeCell ref="N2:Q2"/>
     <mergeCell ref="R2:U2"/>
+    <mergeCell ref="BA1:BE1"/>
+    <mergeCell ref="BA2:BB2"/>
+    <mergeCell ref="BC2:BE2"/>
+    <mergeCell ref="BF1:BM1"/>
+    <mergeCell ref="BF2:BI2"/>
+    <mergeCell ref="BJ2:BM2"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <hyperlinks>
@@ -6450,9 +7317,21 @@
     <hyperlink ref="E35" r:id="rId67" display="https://maniflow-policy.github.io/" xr:uid="{7053B945-7DF7-4C3B-9860-E6888169B40B}"/>
     <hyperlink ref="D36" r:id="rId68" xr:uid="{81E431FC-6990-496A-8A0B-6DBB169E6A58}"/>
     <hyperlink ref="E36" r:id="rId69" xr:uid="{2F7794B4-4E8A-400D-AD7B-9827CFFD7061}"/>
+    <hyperlink ref="D37" r:id="rId70" xr:uid="{71593488-F6AD-4133-9602-8DC98EC6B700}"/>
+    <hyperlink ref="D38" r:id="rId71" xr:uid="{1F931595-1E19-4326-9E56-EE926E639C5E}"/>
+    <hyperlink ref="D39" r:id="rId72" xr:uid="{84BB49A0-6FB4-407E-ABD5-F40679971A87}"/>
+    <hyperlink ref="E39" r:id="rId73" xr:uid="{0FEC1DFC-A1DE-4BA7-A1A2-4AA0BBAFF9A0}"/>
+    <hyperlink ref="D40" r:id="rId74" xr:uid="{75B63F35-D269-405F-AED2-612C785F37C3}"/>
+    <hyperlink ref="E40" r:id="rId75" xr:uid="{97FAB6B1-C35B-4F04-B851-E1A14FDB53F0}"/>
+    <hyperlink ref="D41" r:id="rId76" xr:uid="{82A51CD4-D7E7-4AD1-BCCF-703D5EC34B23}"/>
+    <hyperlink ref="D42" r:id="rId77" xr:uid="{A0067A62-0203-4BDE-A20F-BBA30F0C5DDD}"/>
+    <hyperlink ref="D43" r:id="rId78" xr:uid="{07AC19AB-0CE7-4076-9710-A62A649B43BD}"/>
+    <hyperlink ref="D44" r:id="rId79" xr:uid="{AD4AF1C3-193C-4702-97D1-C608D26EA789}"/>
+    <hyperlink ref="D45" r:id="rId80" xr:uid="{867BDA6D-8529-46A7-9E80-7F92D4A8496F}"/>
+    <hyperlink ref="D46" r:id="rId81" xr:uid="{1905AC21-9861-4EB0-A4AF-C9BEAFD3D922}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId70"/>
-  <drawing r:id="rId71"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId82"/>
+  <drawing r:id="rId83"/>
 </worksheet>
 </file>
</xml_diff>